<commit_message>
Updated Excel sheet with arguments Fixed some comments Added Data driven test from excel
</commit_message>
<xml_diff>
--- a/tests/web/resources/data/login_data.xlsx
+++ b/tests/web/resources/data/login_data.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Source\robotframework-datadriver\example\Login Tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\RobotFramework-Python\tests\web\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{548B6060-6D48-446A-9C04-95DD72398B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC9332C-5468-43CD-94CB-A92EE6AFFAA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38790" yWindow="-2115" windowWidth="21600" windowHeight="11385" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DataDriven" sheetId="1" r:id="rId1"/>
-    <sheet name="2nd Sheet" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>*** Test Cases ***</t>
   </si>
@@ -51,50 +50,56 @@
     <t>[Tags]</t>
   </si>
   <si>
-    <t>[Documentation]</t>
-  </si>
-  <si>
-    <t>Right user empty pass</t>
-  </si>
-  <si>
-    <t>demo</t>
-  </si>
-  <si>
-    <t>${EMPTY}</t>
-  </si>
-  <si>
-    <t>This is a test case documentation of the first one.</t>
-  </si>
-  <si>
-    <t>Right user wrong pass</t>
-  </si>
-  <si>
-    <t>FooBar</t>
-  </si>
-  <si>
-    <t>2,3,foo</t>
-  </si>
-  <si>
-    <t>This test case has the Tags 2,3 and foo</t>
-  </si>
-  <si>
-    <t>mode</t>
-  </si>
-  <si>
-    <t>1,2,3,4</t>
-  </si>
-  <si>
-    <t>This test case has a generated name based on template name.</t>
-  </si>
-  <si>
-    <t>foo</t>
+    <t>${expected_error}</t>
+  </si>
+  <si>
+    <t>Login - Valid Login With Standard User</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>smoke</t>
+  </si>
+  <si>
+    <t>Login - Blank username and password</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username is required</t>
+  </si>
+  <si>
+    <t>negative</t>
+  </si>
+  <si>
+    <t>Login - Valid user Blank password</t>
+  </si>
+  <si>
+    <t>Epic sadface: Password is required</t>
+  </si>
+  <si>
+    <t>regression</t>
+  </si>
+  <si>
+    <t>Login - Incorrect username correct password</t>
+  </si>
+  <si>
+    <t>NotCorrect</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username and password do not match any user in this service</t>
+  </si>
+  <si>
+    <t>Login - Correct username incorrect password</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -228,6 +233,36 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF569CD6"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFDCDCAA"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF6A9955"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="33">
@@ -571,9 +606,24 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -633,9 +683,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -673,7 +723,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -779,7 +829,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -921,7 +971,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -929,287 +979,108 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="56.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
+      <c r="D4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="B4" s="1" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="D5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="B6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="B8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="B9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>16</v>
+      <c r="D6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{271415A9-6699-4C0B-9491-6FAE70C49EF2}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="57.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>